<commit_message>
feat: replace SheetJS with @protobi/exceljs for Excel parsing
Replace the CDN-hosted SheetJS dependency with @protobi/exceljs from npm,
eliminating external CDN dependencies. Drop .xls support (only .xlsx now).
Also self-hosts Inter font via @fontsource, adds unit tests with vitest,
E2E tests, and simplifies CI to use make test.
</commit_message>
<xml_diff>
--- a/v2/e2e/fixtures/test-transactions.xlsx
+++ b/v2/e2e/fixtures/test-transactions.xlsx
@@ -1,47 +1,116 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Transactions" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Transactions" state="visible" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="29">
+  <si>
+    <t>TransactionDate</t>
+  </si>
+  <si>
+    <t>BookDate</t>
+  </si>
+  <si>
+    <t>ValueDate</t>
+  </si>
+  <si>
+    <t>Text</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Currency Amount</t>
+  </si>
+  <si>
+    <t>Currency Rate</t>
+  </si>
+  <si>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Merchant Area</t>
+  </si>
+  <si>
+    <t>Merchant Category</t>
+  </si>
+  <si>
+    <t>2023-03-15</t>
+  </si>
+  <si>
+    <t>Purchase at KOMPLETT.NO - Online</t>
+  </si>
+  <si>
+    <t>Kjøp</t>
+  </si>
+  <si>
+    <t>NOK</t>
+  </si>
+  <si>
+    <t>OSLO</t>
+  </si>
+  <si>
+    <t>Electronic Sales</t>
+  </si>
+  <si>
+    <t>2023-03-20</t>
+  </si>
+  <si>
+    <t>Payment to REMA 1000</t>
+  </si>
+  <si>
+    <t>Grocery Stores, Supermarkets</t>
+  </si>
+  <si>
+    <t>2023-04-02</t>
+  </si>
+  <si>
+    <t>Subscription for NETFLIX</t>
+  </si>
+  <si>
+    <t>2023-04-10</t>
+  </si>
+  <si>
+    <t>ESPRESSO HOUSE</t>
+  </si>
+  <si>
+    <t>Eating places and Restaurants</t>
+  </si>
+  <si>
+    <t>2023-04-15</t>
+  </si>
+  <si>
+    <t>From 123456798012</t>
+  </si>
+  <si>
+    <t>Innbetaling</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -65,13 +134,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,59 +473,60 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>TransactionDate</v>
-      </c>
-      <c r="B1" t="str">
-        <v>BookDate</v>
-      </c>
-      <c r="C1" t="str">
-        <v>ValueDate</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Text</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Type</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Currency Amount</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Currency Rate</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Currency</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Amount</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Merchant Area</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Merchant Category</v>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>2023-03-15</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2023-03-15</v>
-      </c>
-      <c r="C2" t="str">
-        <v>2023-03-15</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Purchase at KOMPLETT.NO - Online</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Kjøp</v>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
       </c>
       <c r="F2">
         <v>-499</v>
@@ -456,34 +534,34 @@
       <c r="G2">
         <v>1</v>
       </c>
-      <c r="H2" t="str">
-        <v>NOK</v>
+      <c r="H2" t="s">
+        <v>14</v>
       </c>
       <c r="I2">
         <v>-499</v>
       </c>
-      <c r="J2" t="str">
-        <v>OSLO</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Electronic Sales</v>
+      <c r="J2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K2" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>2023-03-20</v>
-      </c>
-      <c r="B3" t="str">
-        <v>2023-03-20</v>
-      </c>
-      <c r="C3" t="str">
-        <v>2023-03-20</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Payment to REMA 1000</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Kjøp</v>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
       </c>
       <c r="F3">
         <v>-234.5</v>
@@ -491,34 +569,34 @@
       <c r="G3">
         <v>1</v>
       </c>
-      <c r="H3" t="str">
-        <v>NOK</v>
+      <c r="H3" t="s">
+        <v>14</v>
       </c>
       <c r="I3">
         <v>-234.5</v>
       </c>
-      <c r="J3" t="str">
-        <v>OSLO</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Grocery Stores, Supermarkets</v>
+      <c r="J3" t="s">
+        <v>15</v>
+      </c>
+      <c r="K3" t="s">
+        <v>19</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>2023-04-02</v>
-      </c>
-      <c r="B4" t="str">
-        <v>2023-04-02</v>
-      </c>
-      <c r="C4" t="str">
-        <v>2023-04-02</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Subscription for NETFLIX</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Kjøp</v>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>13</v>
       </c>
       <c r="F4">
         <v>-149</v>
@@ -526,34 +604,34 @@
       <c r="G4">
         <v>1</v>
       </c>
-      <c r="H4" t="str">
-        <v>NOK</v>
+      <c r="H4" t="s">
+        <v>14</v>
       </c>
       <c r="I4">
         <v>-149</v>
       </c>
-      <c r="J4" t="str">
-        <v>OSLO</v>
-      </c>
-      <c r="K4" t="str">
-        <v>Electronic Sales</v>
+      <c r="J4" t="s">
+        <v>15</v>
+      </c>
+      <c r="K4" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>2023-04-10</v>
-      </c>
-      <c r="B5" t="str">
-        <v>2023-04-10</v>
-      </c>
-      <c r="C5" t="str">
-        <v>2023-04-10</v>
-      </c>
-      <c r="D5" t="str">
-        <v>ESPRESSO HOUSE</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Kjøp</v>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
       </c>
       <c r="F5">
         <v>-65</v>
@@ -561,34 +639,34 @@
       <c r="G5">
         <v>1</v>
       </c>
-      <c r="H5" t="str">
-        <v>NOK</v>
+      <c r="H5" t="s">
+        <v>14</v>
       </c>
       <c r="I5">
         <v>-65</v>
       </c>
-      <c r="J5" t="str">
-        <v>OSLO</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Eating places and Restaurants</v>
+      <c r="J5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K5" t="s">
+        <v>24</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>2023-04-15</v>
-      </c>
-      <c r="B6" t="str">
-        <v>2023-04-15</v>
-      </c>
-      <c r="C6" t="str">
-        <v>2023-04-15</v>
-      </c>
-      <c r="D6" t="str">
-        <v>From 123456798012</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Innbetaling</v>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" t="s">
+        <v>27</v>
       </c>
       <c r="F6">
         <v>25000</v>
@@ -596,22 +674,21 @@
       <c r="G6">
         <v>1</v>
       </c>
-      <c r="H6" t="str">
-        <v>NOK</v>
+      <c r="H6" t="s">
+        <v>14</v>
       </c>
       <c r="I6">
         <v>25000</v>
       </c>
-      <c r="J6" t="str">
-        <v/>
-      </c>
-      <c r="K6" t="str">
-        <v/>
+      <c r="J6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Replace SheetJS with @protobi/exceljs (#41)
* feat: replace SheetJS with @protobi/exceljs for Excel parsing

Replace the CDN-hosted SheetJS dependency with @protobi/exceljs from npm,
eliminating external CDN dependencies. Drop .xls support (only .xlsx now).
Also self-hosts Inter font via @fontsource, adds unit tests with vitest,
E2E tests, and simplifies CI to use make test.

* chore: remove tsconfig.tsbuildinfo from git tracking

Already in .gitignore but was previously committed.

* chore: update package-lock.json after rebase

---------

Co-authored-by: User <user@example.com>
</commit_message>
<xml_diff>
--- a/v2/e2e/fixtures/test-transactions.xlsx
+++ b/v2/e2e/fixtures/test-transactions.xlsx
@@ -1,47 +1,116 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Transactions" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Transactions" state="visible" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="29">
+  <si>
+    <t>TransactionDate</t>
+  </si>
+  <si>
+    <t>BookDate</t>
+  </si>
+  <si>
+    <t>ValueDate</t>
+  </si>
+  <si>
+    <t>Text</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Currency Amount</t>
+  </si>
+  <si>
+    <t>Currency Rate</t>
+  </si>
+  <si>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Merchant Area</t>
+  </si>
+  <si>
+    <t>Merchant Category</t>
+  </si>
+  <si>
+    <t>2023-03-15</t>
+  </si>
+  <si>
+    <t>Purchase at KOMPLETT.NO - Online</t>
+  </si>
+  <si>
+    <t>Kjøp</t>
+  </si>
+  <si>
+    <t>NOK</t>
+  </si>
+  <si>
+    <t>OSLO</t>
+  </si>
+  <si>
+    <t>Electronic Sales</t>
+  </si>
+  <si>
+    <t>2023-03-20</t>
+  </si>
+  <si>
+    <t>Payment to REMA 1000</t>
+  </si>
+  <si>
+    <t>Grocery Stores, Supermarkets</t>
+  </si>
+  <si>
+    <t>2023-04-02</t>
+  </si>
+  <si>
+    <t>Subscription for NETFLIX</t>
+  </si>
+  <si>
+    <t>2023-04-10</t>
+  </si>
+  <si>
+    <t>ESPRESSO HOUSE</t>
+  </si>
+  <si>
+    <t>Eating places and Restaurants</t>
+  </si>
+  <si>
+    <t>2023-04-15</t>
+  </si>
+  <si>
+    <t>From 123456798012</t>
+  </si>
+  <si>
+    <t>Innbetaling</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -65,13 +134,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,59 +473,60 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>TransactionDate</v>
-      </c>
-      <c r="B1" t="str">
-        <v>BookDate</v>
-      </c>
-      <c r="C1" t="str">
-        <v>ValueDate</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Text</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Type</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Currency Amount</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Currency Rate</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Currency</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Amount</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Merchant Area</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Merchant Category</v>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>2023-03-15</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2023-03-15</v>
-      </c>
-      <c r="C2" t="str">
-        <v>2023-03-15</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Purchase at KOMPLETT.NO - Online</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Kjøp</v>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
       </c>
       <c r="F2">
         <v>-499</v>
@@ -456,34 +534,34 @@
       <c r="G2">
         <v>1</v>
       </c>
-      <c r="H2" t="str">
-        <v>NOK</v>
+      <c r="H2" t="s">
+        <v>14</v>
       </c>
       <c r="I2">
         <v>-499</v>
       </c>
-      <c r="J2" t="str">
-        <v>OSLO</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Electronic Sales</v>
+      <c r="J2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K2" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>2023-03-20</v>
-      </c>
-      <c r="B3" t="str">
-        <v>2023-03-20</v>
-      </c>
-      <c r="C3" t="str">
-        <v>2023-03-20</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Payment to REMA 1000</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Kjøp</v>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
       </c>
       <c r="F3">
         <v>-234.5</v>
@@ -491,34 +569,34 @@
       <c r="G3">
         <v>1</v>
       </c>
-      <c r="H3" t="str">
-        <v>NOK</v>
+      <c r="H3" t="s">
+        <v>14</v>
       </c>
       <c r="I3">
         <v>-234.5</v>
       </c>
-      <c r="J3" t="str">
-        <v>OSLO</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Grocery Stores, Supermarkets</v>
+      <c r="J3" t="s">
+        <v>15</v>
+      </c>
+      <c r="K3" t="s">
+        <v>19</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>2023-04-02</v>
-      </c>
-      <c r="B4" t="str">
-        <v>2023-04-02</v>
-      </c>
-      <c r="C4" t="str">
-        <v>2023-04-02</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Subscription for NETFLIX</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Kjøp</v>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>13</v>
       </c>
       <c r="F4">
         <v>-149</v>
@@ -526,34 +604,34 @@
       <c r="G4">
         <v>1</v>
       </c>
-      <c r="H4" t="str">
-        <v>NOK</v>
+      <c r="H4" t="s">
+        <v>14</v>
       </c>
       <c r="I4">
         <v>-149</v>
       </c>
-      <c r="J4" t="str">
-        <v>OSLO</v>
-      </c>
-      <c r="K4" t="str">
-        <v>Electronic Sales</v>
+      <c r="J4" t="s">
+        <v>15</v>
+      </c>
+      <c r="K4" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>2023-04-10</v>
-      </c>
-      <c r="B5" t="str">
-        <v>2023-04-10</v>
-      </c>
-      <c r="C5" t="str">
-        <v>2023-04-10</v>
-      </c>
-      <c r="D5" t="str">
-        <v>ESPRESSO HOUSE</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Kjøp</v>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
       </c>
       <c r="F5">
         <v>-65</v>
@@ -561,34 +639,34 @@
       <c r="G5">
         <v>1</v>
       </c>
-      <c r="H5" t="str">
-        <v>NOK</v>
+      <c r="H5" t="s">
+        <v>14</v>
       </c>
       <c r="I5">
         <v>-65</v>
       </c>
-      <c r="J5" t="str">
-        <v>OSLO</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Eating places and Restaurants</v>
+      <c r="J5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K5" t="s">
+        <v>24</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>2023-04-15</v>
-      </c>
-      <c r="B6" t="str">
-        <v>2023-04-15</v>
-      </c>
-      <c r="C6" t="str">
-        <v>2023-04-15</v>
-      </c>
-      <c r="D6" t="str">
-        <v>From 123456798012</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Innbetaling</v>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" t="s">
+        <v>27</v>
       </c>
       <c r="F6">
         <v>25000</v>
@@ -596,22 +674,21 @@
       <c r="G6">
         <v>1</v>
       </c>
-      <c r="H6" t="str">
-        <v>NOK</v>
+      <c r="H6" t="s">
+        <v>14</v>
       </c>
       <c r="I6">
         <v>25000</v>
       </c>
-      <c r="J6" t="str">
-        <v/>
-      </c>
-      <c r="K6" t="str">
-        <v/>
+      <c r="J6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>